<commit_message>
Add parsing functions and constants for crash report fields; enhance value normalization and validation
</commit_message>
<xml_diff>
--- a/outputs/crash_reports.xlsx
+++ b/outputs/crash_reports.xlsx
@@ -427,25 +427,53 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:AR2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="36" customWidth="1" min="10" max="10"/>
-    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
     <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="27" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="36" customWidth="1" min="13" max="13"/>
+    <col width="21" customWidth="1" min="14" max="14"/>
     <col width="15" customWidth="1" min="15" max="15"/>
-    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="17" customWidth="1" min="17" max="17"/>
+    <col width="19" customWidth="1" min="18" max="18"/>
+    <col width="22" customWidth="1" min="19" max="19"/>
+    <col width="27" customWidth="1" min="20" max="20"/>
+    <col width="19" customWidth="1" min="21" max="21"/>
+    <col width="18" customWidth="1" min="22" max="22"/>
+    <col width="34" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="29" customWidth="1" min="25" max="25"/>
+    <col width="16" customWidth="1" min="26" max="26"/>
+    <col width="18" customWidth="1" min="27" max="27"/>
+    <col width="15" customWidth="1" min="28" max="28"/>
+    <col width="14" customWidth="1" min="29" max="29"/>
+    <col width="15" customWidth="1" min="30" max="30"/>
+    <col width="16" customWidth="1" min="31" max="31"/>
+    <col width="17" customWidth="1" min="32" max="32"/>
+    <col width="19" customWidth="1" min="33" max="33"/>
+    <col width="19" customWidth="1" min="34" max="34"/>
+    <col width="20" customWidth="1" min="35" max="35"/>
+    <col width="23" customWidth="1" min="36" max="36"/>
+    <col width="19" customWidth="1" min="37" max="37"/>
+    <col width="23" customWidth="1" min="38" max="38"/>
+    <col width="58" customWidth="1" min="39" max="39"/>
+    <col width="38" customWidth="1" min="40" max="40"/>
+    <col width="64" customWidth="1" min="41" max="41"/>
+    <col width="30" customWidth="1" min="42" max="42"/>
+    <col width="33" customWidth="1" min="43" max="43"/>
+    <col width="32" customWidth="1" min="44" max="44"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -466,67 +494,207 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>station_name</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>investigating_officer</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>severity</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>road_classification</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>road_name</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>collision_type</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>collision_nature</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>traffic_violation</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>weather_condition</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>light_condition</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>accident_spot</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>visibility</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>property_damage</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>damage_value</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>vehicle_reg_no</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>vehicle_type</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>vehicle_category</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>vehicle_class</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>vehicle_color</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>make_model</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>fuel_type</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>vehicle_damage</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>speed_limit</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>driver_gender</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>driver_age</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>speed_limit</t>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>education</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>occupation</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>nationality</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>license_type</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>license_status</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>injury_type</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>brake_condition</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>steering_condition</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>tyre_condition</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>mechanical_failure</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>fir_csr_number</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>state_rule</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>station_address</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>district_code</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>road_details__fir_csr_number</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>road_details__fir_date_time</t>
         </is>
       </c>
     </row>
@@ -548,67 +716,207 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>SVNIT RURAL POLICE</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Harsh Kakkad</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>Fatal</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>National Highway</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>NH 48, SVNIT, Surat</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Vehicle to Pedestrian</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Hit from Side</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
         <is>
           <t>High Speed</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Sunny / Clear</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>Darkness with Poor street light</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Educational Zone</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>100000</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>GJ05MK0000</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
         <is>
           <t>Car/Jeep/Van/Taxi</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>Motorised Fuel Vehicle</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Motor Car(LMV)</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>MIDTOWN_GREY</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>Tata Motors Ltd / Tata Altroz</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>Diesel</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>Front Damage, Top Damage</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
         <is>
           <t>Male</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="AB2" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>100</t>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>Graduate</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>Indian</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>Permanent</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>Satisfactory</t>
+        </is>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>Working</t>
+        </is>
+      </c>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>In Order</t>
+        </is>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>ABC012345678 FIR Date &amp; Time : 20-Jun-2032 : 12:20 PM</t>
+        </is>
+      </c>
+      <c r="AN2" t="inlineStr">
+        <is>
+          <t>NA Accident ID : 2032112233445566</t>
+        </is>
+      </c>
+      <c r="AO2" t="inlineStr">
+        <is>
+          <t>SVNIT, Surat, Gujarat, India Field Officer : Mihir Koladiya</t>
+        </is>
+      </c>
+      <c r="AP2" t="inlineStr">
+        <is>
+          <t>316 District Name : Surat</t>
+        </is>
+      </c>
+      <c r="AQ2" t="inlineStr">
+        <is>
+          <t>ABCO012345678</t>
+        </is>
+      </c>
+      <c r="AR2" t="inlineStr">
+        <is>
+          <t>20-Jun-2032 : 12:20 PM</t>
         </is>
       </c>
     </row>
@@ -623,11 +931,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="33" customWidth="1" min="1" max="1"/>
+    <col width="64" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -681,156 +989,492 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>severity</t>
+          <t>station_name</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Fatal</t>
+          <t>SVNIT RURAL POLICE</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>road_classification</t>
+          <t>investigating_officer</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>National Highway</t>
+          <t>Harsh Kakkad</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>road_name</t>
+          <t>severity</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>NH 48, SVNIT, Surat</t>
+          <t>Fatal</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>collision_type</t>
+          <t>road_classification</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Vehicle to Pedestrian</t>
+          <t>National Highway</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>traffic_violation</t>
+          <t>road_name</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>High Speed</t>
+          <t>NH 48, SVNIT, Surat</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>weather_condition</t>
+          <t>collision_type</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Sunny / Clear</t>
+          <t>Vehicle to Pedestrian</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>light_condition</t>
+          <t>collision_nature</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Darkness with Poor street light</t>
+          <t>Hit from Side</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>accident_spot</t>
+          <t>traffic_violation</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Educational Zone</t>
+          <t>High Speed</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>vehicle_type</t>
+          <t>weather_condition</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Car/Jeep/Van/Taxi</t>
+          <t>Sunny / Clear</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>vehicle_category</t>
+          <t>light_condition</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Motorised Fuel Vehicle</t>
+          <t>Darkness with Poor street light</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>driver_gender</t>
+          <t>accident_spot</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Educational Zone</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>driver_age</t>
+          <t>visibility</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>75</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>property_damage</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>damage_value</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>100000</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>vehicle_reg_no</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>GJ05MK0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>vehicle_type</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Car/Jeep/Van/Taxi</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>vehicle_category</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Motorised Fuel Vehicle</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>vehicle_class</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Motor Car(LMV)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>vehicle_color</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>MIDTOWN_GREY</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>make_model</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Tata Motors Ltd / Tata Altroz</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>fuel_type</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Diesel</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>vehicle_damage</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Front Damage, Top Damage</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>speed_limit</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>100</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>driver_gender</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>driver_age</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>education</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Graduate</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>occupation</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>nationality</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Indian</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>license_type</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Permanent</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>license_status</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>injury_type</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>brake_condition</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Satisfactory</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>steering_condition</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Working</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>tyre_condition</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>In Order</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>mechanical_failure</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>fir_csr_number</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>ABC012345678 FIR Date &amp; Time : 20-Jun-2032 : 12:20 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>state_rule</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>NA Accident ID : 2032112233445566</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>station_address</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>SVNIT, Surat, Gujarat, India Field Officer : Mihir Koladiya</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>district_code</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>316 District Name : Surat</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>road_details__fir_csr_number</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>ABCO012345678</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>road_details__fir_date_time</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>20-Jun-2032 : 12:20 PM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Enhance README with new features and batch processing instructions; refactor parsing logic for improved alias resolution and validation; add batch processing script for handling multiple reports
</commit_message>
<xml_diff>
--- a/outputs/crash_reports.xlsx
+++ b/outputs/crash_reports.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR2"/>
+  <dimension ref="A1:AP2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -468,12 +468,10 @@
     <col width="23" customWidth="1" min="36" max="36"/>
     <col width="19" customWidth="1" min="37" max="37"/>
     <col width="23" customWidth="1" min="38" max="38"/>
-    <col width="58" customWidth="1" min="39" max="39"/>
-    <col width="38" customWidth="1" min="40" max="40"/>
-    <col width="64" customWidth="1" min="41" max="41"/>
-    <col width="30" customWidth="1" min="42" max="42"/>
-    <col width="33" customWidth="1" min="43" max="43"/>
-    <col width="32" customWidth="1" min="44" max="44"/>
+    <col width="38" customWidth="1" min="39" max="39"/>
+    <col width="64" customWidth="1" min="40" max="40"/>
+    <col width="30" customWidth="1" min="41" max="41"/>
+    <col width="32" customWidth="1" min="42" max="42"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -669,30 +667,20 @@
       </c>
       <c r="AM1" s="1" t="inlineStr">
         <is>
-          <t>fir_csr_number</t>
+          <t>state_rule</t>
         </is>
       </c>
       <c r="AN1" s="1" t="inlineStr">
         <is>
-          <t>state_rule</t>
+          <t>station_address</t>
         </is>
       </c>
       <c r="AO1" s="1" t="inlineStr">
         <is>
-          <t>station_address</t>
+          <t>district_code</t>
         </is>
       </c>
       <c r="AP1" s="1" t="inlineStr">
-        <is>
-          <t>district_code</t>
-        </is>
-      </c>
-      <c r="AQ1" s="1" t="inlineStr">
-        <is>
-          <t>road_details__fir_csr_number</t>
-        </is>
-      </c>
-      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>road_details__fir_date_time</t>
         </is>
@@ -891,30 +879,20 @@
       </c>
       <c r="AM2" t="inlineStr">
         <is>
-          <t>ABC012345678 FIR Date &amp; Time : 20-Jun-2032 : 12:20 PM</t>
+          <t>NA Accident ID : 2032112233445566</t>
         </is>
       </c>
       <c r="AN2" t="inlineStr">
         <is>
-          <t>NA Accident ID : 2032112233445566</t>
+          <t>SVNIT, Surat, Gujarat, India Field Officer : Mihir Koladiya</t>
         </is>
       </c>
       <c r="AO2" t="inlineStr">
         <is>
-          <t>SVNIT, Surat, Gujarat, India Field Officer : Mihir Koladiya</t>
+          <t>316 District Name : Surat</t>
         </is>
       </c>
       <c r="AP2" t="inlineStr">
-        <is>
-          <t>316 District Name : Surat</t>
-        </is>
-      </c>
-      <c r="AQ2" t="inlineStr">
-        <is>
-          <t>ABCO012345678</t>
-        </is>
-      </c>
-      <c r="AR2" t="inlineStr">
         <is>
           <t>20-Jun-2032 : 12:20 PM</t>
         </is>
@@ -931,10 +909,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B45"/>
+  <dimension ref="A1:B43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="33" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
     <col width="64" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -1409,70 +1387,46 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>fir_csr_number</t>
+          <t>state_rule</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ABC012345678 FIR Date &amp; Time : 20-Jun-2032 : 12:20 PM</t>
+          <t>NA Accident ID : 2032112233445566</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>state_rule</t>
+          <t>station_address</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>NA Accident ID : 2032112233445566</t>
+          <t>SVNIT, Surat, Gujarat, India Field Officer : Mihir Koladiya</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>station_address</t>
+          <t>district_code</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>SVNIT, Surat, Gujarat, India Field Officer : Mihir Koladiya</t>
+          <t>316 District Name : Surat</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>district_code</t>
+          <t>road_details__fir_date_time</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
-        <is>
-          <t>316 District Name : Surat</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>road_details__fir_csr_number</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>ABCO012345678</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>road_details__fir_date_time</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
         <is>
           <t>20-Jun-2032 : 12:20 PM</t>
         </is>

</xml_diff>